<commit_message>
added folder watcher and auto processing
</commit_message>
<xml_diff>
--- a/timesheets_final.xlsx
+++ b/timesheets_final.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -675,6 +675,190 @@
         <v>5</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>123 Oak Street Residence</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>456 Pine Road - Smith Property</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>123 Oak Street Residence</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>456 Pine Road - Smith Property</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>123 Oak Street Residence</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>456 Pine Road - Smith Property</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>123 Oak Street Residence</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jake Williams</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>04/28/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>456 Pine Road - Smith Property</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>